<commit_message>
Sync Promised Land Cloudbeds export from Drive — 2026-06-29
</commit_message>
<xml_diff>
--- a/PA-PL_occupancy_2026ytd.xlsx
+++ b/PA-PL_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D176"/>
+  <dimension ref="A1:D180"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,13 +432,13 @@
         <v>01/02</v>
       </c>
       <c r="B3">
-        <v>275.09749999999997</v>
+        <v>275.0975</v>
       </c>
       <c r="C3">
         <v>4</v>
       </c>
       <c r="D3">
-        <v>1100.3899999999999</v>
+        <v>1100.39</v>
       </c>
     </row>
     <row r="4">
@@ -1048,13 +1048,13 @@
         <v>02/15</v>
       </c>
       <c r="B47">
-        <v>326.5983333333333</v>
+        <v>326.59833333333336</v>
       </c>
       <c r="C47">
         <v>6</v>
       </c>
       <c r="D47">
-        <v>1959.59</v>
+        <v>1959.5900000000001</v>
       </c>
     </row>
     <row r="48">
@@ -1124,7 +1124,7 @@
         <v>5</v>
       </c>
       <c r="D52">
-        <v>1290.6499999999999</v>
+        <v>1290.65</v>
       </c>
     </row>
     <row r="53">
@@ -1132,13 +1132,13 @@
         <v>02/21</v>
       </c>
       <c r="B53">
-        <v>266.468</v>
+        <v>266.46799999999996</v>
       </c>
       <c r="C53">
         <v>5</v>
       </c>
       <c r="D53">
-        <v>1332.3400000000001</v>
+        <v>1332.34</v>
       </c>
     </row>
     <row r="54">
@@ -1608,13 +1608,13 @@
         <v>03/27</v>
       </c>
       <c r="B87">
-        <v>181.83999999999997</v>
+        <v>181.84</v>
       </c>
       <c r="C87">
         <v>5</v>
       </c>
       <c r="D87">
-        <v>909.1999999999999</v>
+        <v>909.2</v>
       </c>
     </row>
     <row r="88">
@@ -1678,13 +1678,13 @@
         <v>04/01</v>
       </c>
       <c r="B92">
-        <v>165.86666666666667</v>
+        <v>165.86666666666665</v>
       </c>
       <c r="C92">
         <v>6</v>
       </c>
       <c r="D92">
-        <v>995.2</v>
+        <v>995.1999999999999</v>
       </c>
     </row>
     <row r="93">
@@ -2112,13 +2112,13 @@
         <v>05/02</v>
       </c>
       <c r="B123">
-        <v>236.94285714285715</v>
+        <v>236.94285714285712</v>
       </c>
       <c r="C123">
         <v>14</v>
       </c>
       <c r="D123">
-        <v>3317.2000000000003</v>
+        <v>3317.2</v>
       </c>
     </row>
     <row r="124">
@@ -2322,13 +2322,13 @@
         <v>05/17</v>
       </c>
       <c r="B138">
-        <v>187.57500000000002</v>
+        <v>187.575</v>
       </c>
       <c r="C138">
         <v>8</v>
       </c>
       <c r="D138">
-        <v>1500.6000000000001</v>
+        <v>1500.6</v>
       </c>
     </row>
     <row r="139">
@@ -2398,7 +2398,7 @@
         <v>12</v>
       </c>
       <c r="D143">
-        <v>3448.4500000000003</v>
+        <v>3448.45</v>
       </c>
     </row>
     <row r="144">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>283.97772727272724</v>
+        <v>283.9777272727272</v>
       </c>
       <c r="C144">
         <v>22</v>
       </c>
       <c r="D144">
-        <v>6247.509999999999</v>
+        <v>6247.509999999998</v>
       </c>
     </row>
     <row r="145">
@@ -2420,13 +2420,13 @@
         <v>05/24</v>
       </c>
       <c r="B145">
-        <v>294.62590909090903</v>
+        <v>294.6259090909091</v>
       </c>
       <c r="C145">
         <v>22</v>
       </c>
       <c r="D145">
-        <v>6481.769999999999</v>
+        <v>6481.7699999999995</v>
       </c>
     </row>
     <row r="146">
@@ -2434,13 +2434,13 @@
         <v>05/25</v>
       </c>
       <c r="B146">
-        <v>177.4811111111111</v>
+        <v>177.48111111111112</v>
       </c>
       <c r="C146">
         <v>9</v>
       </c>
       <c r="D146">
-        <v>1597.33</v>
+        <v>1597.3300000000002</v>
       </c>
     </row>
     <row r="147">
@@ -2588,13 +2588,13 @@
         <v>06/05</v>
       </c>
       <c r="B157">
-        <v>253.39499999999998</v>
+        <v>253.39499999999995</v>
       </c>
       <c r="C157">
         <v>16</v>
       </c>
       <c r="D157">
-        <v>4054.3199999999997</v>
+        <v>4054.3199999999993</v>
       </c>
     </row>
     <row r="158">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>276.4234782608696</v>
+        <v>276.4234782608695</v>
       </c>
       <c r="C165">
         <v>23</v>
       </c>
       <c r="D165">
-        <v>6357.740000000001</v>
+        <v>6357.739999999999</v>
       </c>
     </row>
     <row r="166">
@@ -2714,13 +2714,13 @@
         <v>06/14</v>
       </c>
       <c r="B166">
-        <v>224.31833333333336</v>
+        <v>224.3183333333333</v>
       </c>
       <c r="C166">
         <v>6</v>
       </c>
       <c r="D166">
-        <v>1345.91</v>
+        <v>1345.9099999999999</v>
       </c>
     </row>
     <row r="167">
@@ -2770,13 +2770,13 @@
         <v>06/18</v>
       </c>
       <c r="B170">
-        <v>234.69636363636363</v>
+        <v>234.69636363636366</v>
       </c>
       <c r="C170">
         <v>11</v>
       </c>
       <c r="D170">
-        <v>2581.66</v>
+        <v>2581.6600000000003</v>
       </c>
     </row>
     <row r="171">
@@ -2804,7 +2804,7 @@
         <v>19</v>
       </c>
       <c r="D172">
-        <v>6173.47</v>
+        <v>6173.469999999999</v>
       </c>
     </row>
     <row r="173">
@@ -2863,9 +2863,65 @@
         <v>932.8</v>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>06/25</v>
+      </c>
+      <c r="B177">
+        <v>263</v>
+      </c>
+      <c r="C177">
+        <v>3</v>
+      </c>
+      <c r="D177">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>06/26</v>
+      </c>
+      <c r="B178">
+        <v>300.41249999999997</v>
+      </c>
+      <c r="C178">
+        <v>16</v>
+      </c>
+      <c r="D178">
+        <v>4806.599999999999</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>06/27</v>
+      </c>
+      <c r="B179">
+        <v>305.4854545454546</v>
+      </c>
+      <c r="C179">
+        <v>22</v>
+      </c>
+      <c r="D179">
+        <v>6720.680000000001</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>06/28</v>
+      </c>
+      <c r="B180">
+        <v>253.67071428571427</v>
+      </c>
+      <c r="C180">
+        <v>14</v>
+      </c>
+      <c r="D180">
+        <v>3551.39</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D176"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D180"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Promised Land Cloudbeds export from Drive — 2026-07-06
</commit_message>
<xml_diff>
--- a/PA-PL_occupancy_2026ytd.xlsx
+++ b/PA-PL_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D180"/>
+  <dimension ref="A1:D187"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,13 +432,13 @@
         <v>01/02</v>
       </c>
       <c r="B3">
-        <v>275.0975</v>
+        <v>275.09749999999997</v>
       </c>
       <c r="C3">
         <v>4</v>
       </c>
       <c r="D3">
-        <v>1100.39</v>
+        <v>1100.3899999999999</v>
       </c>
     </row>
     <row r="4">
@@ -642,13 +642,13 @@
         <v>01/17</v>
       </c>
       <c r="B18">
-        <v>300.9666666666667</v>
+        <v>300.96666666666664</v>
       </c>
       <c r="C18">
         <v>6</v>
       </c>
       <c r="D18">
-        <v>1805.8000000000002</v>
+        <v>1805.8</v>
       </c>
     </row>
     <row r="19">
@@ -1132,13 +1132,13 @@
         <v>02/21</v>
       </c>
       <c r="B53">
-        <v>266.46799999999996</v>
+        <v>266.468</v>
       </c>
       <c r="C53">
         <v>5</v>
       </c>
       <c r="D53">
-        <v>1332.34</v>
+        <v>1332.3400000000001</v>
       </c>
     </row>
     <row r="54">
@@ -1608,13 +1608,13 @@
         <v>03/27</v>
       </c>
       <c r="B87">
-        <v>181.84</v>
+        <v>181.83999999999997</v>
       </c>
       <c r="C87">
         <v>5</v>
       </c>
       <c r="D87">
-        <v>909.2</v>
+        <v>909.1999999999999</v>
       </c>
     </row>
     <row r="88">
@@ -1670,7 +1670,7 @@
         <v>6</v>
       </c>
       <c r="D91">
-        <v>1023.5999999999999</v>
+        <v>1023.6</v>
       </c>
     </row>
     <row r="92">
@@ -1902,13 +1902,13 @@
         <v>04/17</v>
       </c>
       <c r="B108">
-        <v>210.77142857142857</v>
+        <v>210.77142857142854</v>
       </c>
       <c r="C108">
         <v>14</v>
       </c>
       <c r="D108">
-        <v>2950.8</v>
+        <v>2950.7999999999997</v>
       </c>
     </row>
     <row r="109">
@@ -2000,13 +2000,13 @@
         <v>04/24</v>
       </c>
       <c r="B115">
-        <v>206.55000000000004</v>
+        <v>206.54999999999998</v>
       </c>
       <c r="C115">
         <v>12</v>
       </c>
       <c r="D115">
-        <v>2478.6000000000004</v>
+        <v>2478.6</v>
       </c>
     </row>
     <row r="116">
@@ -2210,13 +2210,13 @@
         <v>05/09</v>
       </c>
       <c r="B130">
-        <v>288.525</v>
+        <v>288.52500000000003</v>
       </c>
       <c r="C130">
         <v>8</v>
       </c>
       <c r="D130">
-        <v>2308.2</v>
+        <v>2308.2000000000003</v>
       </c>
     </row>
     <row r="131">
@@ -2322,13 +2322,13 @@
         <v>05/17</v>
       </c>
       <c r="B138">
-        <v>187.575</v>
+        <v>187.57500000000002</v>
       </c>
       <c r="C138">
         <v>8</v>
       </c>
       <c r="D138">
-        <v>1500.6</v>
+        <v>1500.6000000000001</v>
       </c>
     </row>
     <row r="139">
@@ -2398,7 +2398,7 @@
         <v>12</v>
       </c>
       <c r="D143">
-        <v>3448.45</v>
+        <v>3448.4500000000003</v>
       </c>
     </row>
     <row r="144">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>283.9777272727272</v>
+        <v>283.97772727272724</v>
       </c>
       <c r="C144">
         <v>22</v>
       </c>
       <c r="D144">
-        <v>6247.509999999998</v>
+        <v>6247.509999999999</v>
       </c>
     </row>
     <row r="145">
@@ -2420,13 +2420,13 @@
         <v>05/24</v>
       </c>
       <c r="B145">
-        <v>294.6259090909091</v>
+        <v>294.62590909090903</v>
       </c>
       <c r="C145">
         <v>22</v>
       </c>
       <c r="D145">
-        <v>6481.7699999999995</v>
+        <v>6481.769999999999</v>
       </c>
     </row>
     <row r="146">
@@ -2434,13 +2434,13 @@
         <v>05/25</v>
       </c>
       <c r="B146">
-        <v>177.48111111111112</v>
+        <v>177.4811111111111</v>
       </c>
       <c r="C146">
         <v>9</v>
       </c>
       <c r="D146">
-        <v>1597.3300000000002</v>
+        <v>1597.33</v>
       </c>
     </row>
     <row r="147">
@@ -2504,13 +2504,13 @@
         <v>05/30</v>
       </c>
       <c r="B151">
-        <v>274.6676470588235</v>
+        <v>274.66764705882355</v>
       </c>
       <c r="C151">
         <v>17</v>
       </c>
       <c r="D151">
-        <v>4669.349999999999</v>
+        <v>4669.35</v>
       </c>
     </row>
     <row r="152">
@@ -2588,13 +2588,13 @@
         <v>06/05</v>
       </c>
       <c r="B157">
-        <v>253.39499999999995</v>
+        <v>253.39499999999998</v>
       </c>
       <c r="C157">
         <v>16</v>
       </c>
       <c r="D157">
-        <v>4054.3199999999993</v>
+        <v>4054.3199999999997</v>
       </c>
     </row>
     <row r="158">
@@ -2602,13 +2602,13 @@
         <v>06/06</v>
       </c>
       <c r="B158">
-        <v>270.34882352941173</v>
+        <v>270.3488235294118</v>
       </c>
       <c r="C158">
         <v>17</v>
       </c>
       <c r="D158">
-        <v>4595.929999999999</v>
+        <v>4595.93</v>
       </c>
     </row>
     <row r="159">
@@ -2686,13 +2686,13 @@
         <v>06/12</v>
       </c>
       <c r="B164">
-        <v>268.81588235294123</v>
+        <v>268.8158823529412</v>
       </c>
       <c r="C164">
         <v>17</v>
       </c>
       <c r="D164">
-        <v>4569.870000000001</v>
+        <v>4569.87</v>
       </c>
     </row>
     <row r="165">
@@ -2714,13 +2714,13 @@
         <v>06/14</v>
       </c>
       <c r="B166">
-        <v>224.3183333333333</v>
+        <v>224.31833333333336</v>
       </c>
       <c r="C166">
         <v>6</v>
       </c>
       <c r="D166">
-        <v>1345.9099999999999</v>
+        <v>1345.91</v>
       </c>
     </row>
     <row r="167">
@@ -2770,13 +2770,13 @@
         <v>06/18</v>
       </c>
       <c r="B170">
-        <v>234.69636363636366</v>
+        <v>234.69636363636363</v>
       </c>
       <c r="C170">
         <v>11</v>
       </c>
       <c r="D170">
-        <v>2581.6600000000003</v>
+        <v>2581.66</v>
       </c>
     </row>
     <row r="171">
@@ -2882,13 +2882,13 @@
         <v>06/26</v>
       </c>
       <c r="B178">
-        <v>300.41249999999997</v>
+        <v>300.4125</v>
       </c>
       <c r="C178">
         <v>16</v>
       </c>
       <c r="D178">
-        <v>4806.599999999999</v>
+        <v>4806.6</v>
       </c>
     </row>
     <row r="179">
@@ -2910,18 +2910,116 @@
         <v>06/28</v>
       </c>
       <c r="B180">
-        <v>253.67071428571427</v>
+        <v>253.6707142857143</v>
       </c>
       <c r="C180">
         <v>14</v>
       </c>
       <c r="D180">
-        <v>3551.39</v>
+        <v>3551.3900000000003</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>06/29</v>
+      </c>
+      <c r="B181">
+        <v>241.59375</v>
+      </c>
+      <c r="C181">
+        <v>8</v>
+      </c>
+      <c r="D181">
+        <v>1932.75</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>06/30</v>
+      </c>
+      <c r="B182">
+        <v>276.6775</v>
+      </c>
+      <c r="C182">
+        <v>4</v>
+      </c>
+      <c r="D182">
+        <v>1106.71</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>07/01</v>
+      </c>
+      <c r="B183">
+        <v>275.57444444444445</v>
+      </c>
+      <c r="C183">
+        <v>9</v>
+      </c>
+      <c r="D183">
+        <v>2480.17</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>07/02</v>
+      </c>
+      <c r="B184">
+        <v>346.90500000000003</v>
+      </c>
+      <c r="C184">
+        <v>6</v>
+      </c>
+      <c r="D184">
+        <v>2081.4300000000003</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>07/03</v>
+      </c>
+      <c r="B185">
+        <v>437.1463636363636</v>
+      </c>
+      <c r="C185">
+        <v>22</v>
+      </c>
+      <c r="D185">
+        <v>9617.22</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>07/04</v>
+      </c>
+      <c r="B186">
+        <v>408.35521739130434</v>
+      </c>
+      <c r="C186">
+        <v>23</v>
+      </c>
+      <c r="D186">
+        <v>9392.17</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>07/05</v>
+      </c>
+      <c r="B187">
+        <v>218.89300000000003</v>
+      </c>
+      <c r="C187">
+        <v>10</v>
+      </c>
+      <c r="D187">
+        <v>2188.9300000000003</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D180"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D187"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Promised Land Cloudbeds export from Drive — 2026-07-13
</commit_message>
<xml_diff>
--- a/PA-PL_occupancy_2026ytd.xlsx
+++ b/PA-PL_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D187"/>
+  <dimension ref="A1:D194"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -572,13 +572,13 @@
         <v>01/12</v>
       </c>
       <c r="B13">
-        <v>122.93333333333332</v>
+        <v>122.93333333333334</v>
       </c>
       <c r="C13">
         <v>3</v>
       </c>
       <c r="D13">
-        <v>368.79999999999995</v>
+        <v>368.8</v>
       </c>
     </row>
     <row r="14">
@@ -1230,13 +1230,13 @@
         <v>02/28</v>
       </c>
       <c r="B60">
-        <v>239.05333333333337</v>
+        <v>239.0533333333333</v>
       </c>
       <c r="C60">
         <v>6</v>
       </c>
       <c r="D60">
-        <v>1434.3200000000002</v>
+        <v>1434.32</v>
       </c>
     </row>
     <row r="61">
@@ -1412,13 +1412,13 @@
         <v>03/13</v>
       </c>
       <c r="B73">
-        <v>200.87</v>
+        <v>200.86999999999998</v>
       </c>
       <c r="C73">
         <v>6</v>
       </c>
       <c r="D73">
-        <v>1205.22</v>
+        <v>1205.2199999999998</v>
       </c>
     </row>
     <row r="74">
@@ -1670,7 +1670,7 @@
         <v>6</v>
       </c>
       <c r="D91">
-        <v>1023.6</v>
+        <v>1023.5999999999999</v>
       </c>
     </row>
     <row r="92">
@@ -1902,13 +1902,13 @@
         <v>04/17</v>
       </c>
       <c r="B108">
-        <v>210.77142857142854</v>
+        <v>210.77142857142857</v>
       </c>
       <c r="C108">
         <v>14</v>
       </c>
       <c r="D108">
-        <v>2950.7999999999997</v>
+        <v>2950.8</v>
       </c>
     </row>
     <row r="109">
@@ -2210,13 +2210,13 @@
         <v>05/09</v>
       </c>
       <c r="B130">
-        <v>288.52500000000003</v>
+        <v>288.525</v>
       </c>
       <c r="C130">
         <v>8</v>
       </c>
       <c r="D130">
-        <v>2308.2000000000003</v>
+        <v>2308.2</v>
       </c>
     </row>
     <row r="131">
@@ -2294,13 +2294,13 @@
         <v>05/15</v>
       </c>
       <c r="B136">
-        <v>287.18666666666667</v>
+        <v>287.1866666666667</v>
       </c>
       <c r="C136">
         <v>15</v>
       </c>
       <c r="D136">
-        <v>4307.8</v>
+        <v>4307.800000000001</v>
       </c>
     </row>
     <row r="137">
@@ -2350,13 +2350,13 @@
         <v>05/19</v>
       </c>
       <c r="B140">
-        <v>141.275</v>
+        <v>141.27499999999998</v>
       </c>
       <c r="C140">
         <v>8</v>
       </c>
       <c r="D140">
-        <v>1130.2</v>
+        <v>1130.1999999999998</v>
       </c>
     </row>
     <row r="141">
@@ -2398,7 +2398,7 @@
         <v>12</v>
       </c>
       <c r="D143">
-        <v>3448.4500000000003</v>
+        <v>3448.45</v>
       </c>
     </row>
     <row r="144">
@@ -2420,13 +2420,13 @@
         <v>05/24</v>
       </c>
       <c r="B145">
-        <v>294.62590909090903</v>
+        <v>294.6259090909091</v>
       </c>
       <c r="C145">
         <v>22</v>
       </c>
       <c r="D145">
-        <v>6481.769999999999</v>
+        <v>6481.7699999999995</v>
       </c>
     </row>
     <row r="146">
@@ -2518,13 +2518,13 @@
         <v>05/31</v>
       </c>
       <c r="B152">
-        <v>209.8222222222222</v>
+        <v>209.82222222222222</v>
       </c>
       <c r="C152">
         <v>9</v>
       </c>
       <c r="D152">
-        <v>1888.3999999999999</v>
+        <v>1888.4</v>
       </c>
     </row>
     <row r="153">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>276.4234782608695</v>
+        <v>276.42347826086956</v>
       </c>
       <c r="C165">
         <v>23</v>
       </c>
       <c r="D165">
-        <v>6357.739999999999</v>
+        <v>6357.74</v>
       </c>
     </row>
     <row r="166">
@@ -2790,7 +2790,7 @@
         <v>19</v>
       </c>
       <c r="D171">
-        <v>5804.25</v>
+        <v>5804.250000000001</v>
       </c>
     </row>
     <row r="172">
@@ -2840,13 +2840,13 @@
         <v>06/23</v>
       </c>
       <c r="B175">
-        <v>232.0233333333333</v>
+        <v>232.02333333333334</v>
       </c>
       <c r="C175">
         <v>6</v>
       </c>
       <c r="D175">
-        <v>1392.1399999999999</v>
+        <v>1392.14</v>
       </c>
     </row>
     <row r="176">
@@ -2882,13 +2882,13 @@
         <v>06/26</v>
       </c>
       <c r="B178">
-        <v>300.4125</v>
+        <v>300.41249999999997</v>
       </c>
       <c r="C178">
         <v>16</v>
       </c>
       <c r="D178">
-        <v>4806.6</v>
+        <v>4806.599999999999</v>
       </c>
     </row>
     <row r="179">
@@ -2896,13 +2896,13 @@
         <v>06/27</v>
       </c>
       <c r="B179">
-        <v>305.4854545454546</v>
+        <v>305.4854545454545</v>
       </c>
       <c r="C179">
         <v>22</v>
       </c>
       <c r="D179">
-        <v>6720.680000000001</v>
+        <v>6720.679999999999</v>
       </c>
     </row>
     <row r="180">
@@ -2910,13 +2910,13 @@
         <v>06/28</v>
       </c>
       <c r="B180">
-        <v>253.6707142857143</v>
+        <v>253.67071428571427</v>
       </c>
       <c r="C180">
         <v>14</v>
       </c>
       <c r="D180">
-        <v>3551.3900000000003</v>
+        <v>3551.39</v>
       </c>
     </row>
     <row r="181">
@@ -2966,13 +2966,13 @@
         <v>07/02</v>
       </c>
       <c r="B184">
-        <v>346.90500000000003</v>
+        <v>346.905</v>
       </c>
       <c r="C184">
         <v>6</v>
       </c>
       <c r="D184">
-        <v>2081.4300000000003</v>
+        <v>2081.43</v>
       </c>
     </row>
     <row r="185">
@@ -2980,13 +2980,13 @@
         <v>07/03</v>
       </c>
       <c r="B185">
-        <v>437.1463636363636</v>
+        <v>437.1463636363637</v>
       </c>
       <c r="C185">
         <v>22</v>
       </c>
       <c r="D185">
-        <v>9617.22</v>
+        <v>9617.220000000001</v>
       </c>
     </row>
     <row r="186">
@@ -3017,9 +3017,107 @@
         <v>2188.9300000000003</v>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>07/06</v>
+      </c>
+      <c r="B188">
+        <v>228.15</v>
+      </c>
+      <c r="C188">
+        <v>8</v>
+      </c>
+      <c r="D188">
+        <v>1825.2</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>07/07</v>
+      </c>
+      <c r="B189">
+        <v>213.58500000000004</v>
+      </c>
+      <c r="C189">
+        <v>10</v>
+      </c>
+      <c r="D189">
+        <v>2135.8500000000004</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>07/08</v>
+      </c>
+      <c r="B190">
+        <v>213.252</v>
+      </c>
+      <c r="C190">
+        <v>5</v>
+      </c>
+      <c r="D190">
+        <v>1066.26</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>07/09</v>
+      </c>
+      <c r="B191">
+        <v>247.2444444444444</v>
+      </c>
+      <c r="C191">
+        <v>9</v>
+      </c>
+      <c r="D191">
+        <v>2225.2</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>07/10</v>
+      </c>
+      <c r="B192">
+        <v>350.13352941176475</v>
+      </c>
+      <c r="C192">
+        <v>17</v>
+      </c>
+      <c r="D192">
+        <v>5952.27</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>07/11</v>
+      </c>
+      <c r="B193">
+        <v>335.62952380952385</v>
+      </c>
+      <c r="C193">
+        <v>21</v>
+      </c>
+      <c r="D193">
+        <v>7048.22</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>07/12</v>
+      </c>
+      <c r="B194">
+        <v>250.16125</v>
+      </c>
+      <c r="C194">
+        <v>8</v>
+      </c>
+      <c r="D194">
+        <v>2001.29</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D187"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D194"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Promised Land Cloudbeds export from Drive — 2026-07-27
</commit_message>
<xml_diff>
--- a/PA-PL_occupancy_2026ytd.xlsx
+++ b/PA-PL_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D194"/>
+  <dimension ref="A1:D208"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -572,13 +572,13 @@
         <v>01/12</v>
       </c>
       <c r="B13">
-        <v>122.93333333333334</v>
+        <v>122.93333333333332</v>
       </c>
       <c r="C13">
         <v>3</v>
       </c>
       <c r="D13">
-        <v>368.8</v>
+        <v>368.79999999999995</v>
       </c>
     </row>
     <row r="14">
@@ -1132,13 +1132,13 @@
         <v>02/21</v>
       </c>
       <c r="B53">
-        <v>266.468</v>
+        <v>266.46799999999996</v>
       </c>
       <c r="C53">
         <v>5</v>
       </c>
       <c r="D53">
-        <v>1332.3400000000001</v>
+        <v>1332.34</v>
       </c>
     </row>
     <row r="54">
@@ -1678,13 +1678,13 @@
         <v>04/01</v>
       </c>
       <c r="B92">
-        <v>165.86666666666665</v>
+        <v>165.86666666666667</v>
       </c>
       <c r="C92">
         <v>6</v>
       </c>
       <c r="D92">
-        <v>995.1999999999999</v>
+        <v>995.2</v>
       </c>
     </row>
     <row r="93">
@@ -2000,13 +2000,13 @@
         <v>04/24</v>
       </c>
       <c r="B115">
-        <v>206.54999999999998</v>
+        <v>206.55000000000004</v>
       </c>
       <c r="C115">
         <v>12</v>
       </c>
       <c r="D115">
-        <v>2478.6</v>
+        <v>2478.6000000000004</v>
       </c>
     </row>
     <row r="116">
@@ -2294,13 +2294,13 @@
         <v>05/15</v>
       </c>
       <c r="B136">
-        <v>287.1866666666667</v>
+        <v>287.18666666666667</v>
       </c>
       <c r="C136">
         <v>15</v>
       </c>
       <c r="D136">
-        <v>4307.800000000001</v>
+        <v>4307.8</v>
       </c>
     </row>
     <row r="137">
@@ -2322,13 +2322,13 @@
         <v>05/17</v>
       </c>
       <c r="B138">
-        <v>187.57500000000002</v>
+        <v>187.575</v>
       </c>
       <c r="C138">
         <v>8</v>
       </c>
       <c r="D138">
-        <v>1500.6000000000001</v>
+        <v>1500.6</v>
       </c>
     </row>
     <row r="139">
@@ -2398,7 +2398,7 @@
         <v>12</v>
       </c>
       <c r="D143">
-        <v>3448.45</v>
+        <v>3448.4500000000003</v>
       </c>
     </row>
     <row r="144">
@@ -2420,13 +2420,13 @@
         <v>05/24</v>
       </c>
       <c r="B145">
-        <v>294.6259090909091</v>
+        <v>294.62590909090903</v>
       </c>
       <c r="C145">
         <v>22</v>
       </c>
       <c r="D145">
-        <v>6481.7699999999995</v>
+        <v>6481.769999999999</v>
       </c>
     </row>
     <row r="146">
@@ -2518,13 +2518,13 @@
         <v>05/31</v>
       </c>
       <c r="B152">
-        <v>209.82222222222222</v>
+        <v>209.8222222222222</v>
       </c>
       <c r="C152">
         <v>9</v>
       </c>
       <c r="D152">
-        <v>1888.4</v>
+        <v>1888.3999999999999</v>
       </c>
     </row>
     <row r="153">
@@ -2588,13 +2588,13 @@
         <v>06/05</v>
       </c>
       <c r="B157">
-        <v>253.39499999999998</v>
+        <v>253.39499999999995</v>
       </c>
       <c r="C157">
         <v>16</v>
       </c>
       <c r="D157">
-        <v>4054.3199999999997</v>
+        <v>4054.3199999999993</v>
       </c>
     </row>
     <row r="158">
@@ -2602,13 +2602,13 @@
         <v>06/06</v>
       </c>
       <c r="B158">
-        <v>270.3488235294118</v>
+        <v>270.34882352941173</v>
       </c>
       <c r="C158">
         <v>17</v>
       </c>
       <c r="D158">
-        <v>4595.93</v>
+        <v>4595.929999999999</v>
       </c>
     </row>
     <row r="159">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>276.42347826086956</v>
+        <v>276.4234782608696</v>
       </c>
       <c r="C165">
         <v>23</v>
       </c>
       <c r="D165">
-        <v>6357.74</v>
+        <v>6357.740000000001</v>
       </c>
     </row>
     <row r="166">
@@ -2714,13 +2714,13 @@
         <v>06/14</v>
       </c>
       <c r="B166">
-        <v>224.31833333333336</v>
+        <v>224.3183333333333</v>
       </c>
       <c r="C166">
         <v>6</v>
       </c>
       <c r="D166">
-        <v>1345.91</v>
+        <v>1345.9099999999999</v>
       </c>
     </row>
     <row r="167">
@@ -2790,7 +2790,7 @@
         <v>19</v>
       </c>
       <c r="D171">
-        <v>5804.250000000001</v>
+        <v>5804.25</v>
       </c>
     </row>
     <row r="172">
@@ -2812,13 +2812,13 @@
         <v>06/21</v>
       </c>
       <c r="B173">
-        <v>199.65333333333334</v>
+        <v>199.6533333333333</v>
       </c>
       <c r="C173">
         <v>15</v>
       </c>
       <c r="D173">
-        <v>2994.8</v>
+        <v>2994.7999999999997</v>
       </c>
     </row>
     <row r="174">
@@ -2882,13 +2882,13 @@
         <v>06/26</v>
       </c>
       <c r="B178">
-        <v>300.41249999999997</v>
+        <v>300.4125</v>
       </c>
       <c r="C178">
         <v>16</v>
       </c>
       <c r="D178">
-        <v>4806.599999999999</v>
+        <v>4806.6</v>
       </c>
     </row>
     <row r="179">
@@ -2896,13 +2896,13 @@
         <v>06/27</v>
       </c>
       <c r="B179">
-        <v>305.4854545454545</v>
+        <v>305.48545454545456</v>
       </c>
       <c r="C179">
         <v>22</v>
       </c>
       <c r="D179">
-        <v>6720.679999999999</v>
+        <v>6720.68</v>
       </c>
     </row>
     <row r="180">
@@ -2980,13 +2980,13 @@
         <v>07/03</v>
       </c>
       <c r="B185">
-        <v>437.1463636363637</v>
+        <v>437.1463636363636</v>
       </c>
       <c r="C185">
         <v>22</v>
       </c>
       <c r="D185">
-        <v>9617.220000000001</v>
+        <v>9617.22</v>
       </c>
     </row>
     <row r="186">
@@ -3036,13 +3036,13 @@
         <v>07/07</v>
       </c>
       <c r="B189">
-        <v>213.58500000000004</v>
+        <v>213.58499999999998</v>
       </c>
       <c r="C189">
         <v>10</v>
       </c>
       <c r="D189">
-        <v>2135.8500000000004</v>
+        <v>2135.85</v>
       </c>
     </row>
     <row r="190">
@@ -3115,9 +3115,205 @@
         <v>2001.29</v>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>07/13</v>
+      </c>
+      <c r="B195">
+        <v>242.96599999999998</v>
+      </c>
+      <c r="C195">
+        <v>5</v>
+      </c>
+      <c r="D195">
+        <v>1214.83</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>07/14</v>
+      </c>
+      <c r="B196">
+        <v>190.66750000000002</v>
+      </c>
+      <c r="C196">
+        <v>4</v>
+      </c>
+      <c r="D196">
+        <v>762.6700000000001</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>07/15</v>
+      </c>
+      <c r="B197">
+        <v>68.79916666666666</v>
+      </c>
+      <c r="C197">
+        <v>12</v>
+      </c>
+      <c r="D197">
+        <v>825.5899999999999</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>07/16</v>
+      </c>
+      <c r="B198">
+        <v>222.03166666666667</v>
+      </c>
+      <c r="C198">
+        <v>6</v>
+      </c>
+      <c r="D198">
+        <v>1332.19</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>07/17</v>
+      </c>
+      <c r="B199">
+        <v>318.5835294117647</v>
+      </c>
+      <c r="C199">
+        <v>17</v>
+      </c>
+      <c r="D199">
+        <v>5415.92</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>07/18</v>
+      </c>
+      <c r="B200">
+        <v>311.26523809523815</v>
+      </c>
+      <c r="C200">
+        <v>21</v>
+      </c>
+      <c r="D200">
+        <v>6536.570000000001</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>07/19</v>
+      </c>
+      <c r="B201">
+        <v>269.0576923076923</v>
+      </c>
+      <c r="C201">
+        <v>13</v>
+      </c>
+      <c r="D201">
+        <v>3497.75</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>07/20</v>
+      </c>
+      <c r="B202">
+        <v>262.5777777777778</v>
+      </c>
+      <c r="C202">
+        <v>9</v>
+      </c>
+      <c r="D202">
+        <v>2363.2</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>07/21</v>
+      </c>
+      <c r="B203">
+        <v>294.09</v>
+      </c>
+      <c r="C203">
+        <v>6</v>
+      </c>
+      <c r="D203">
+        <v>1764.54</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>07/22</v>
+      </c>
+      <c r="B204">
+        <v>217.68666666666664</v>
+      </c>
+      <c r="C204">
+        <v>6</v>
+      </c>
+      <c r="D204">
+        <v>1306.12</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>07/23</v>
+      </c>
+      <c r="B205">
+        <v>227.63666666666668</v>
+      </c>
+      <c r="C205">
+        <v>6</v>
+      </c>
+      <c r="D205">
+        <v>1365.8200000000002</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>07/24</v>
+      </c>
+      <c r="B206">
+        <v>292.4472727272727</v>
+      </c>
+      <c r="C206">
+        <v>22</v>
+      </c>
+      <c r="D206">
+        <v>6433.84</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>07/25</v>
+      </c>
+      <c r="B207">
+        <v>299.43708333333336</v>
+      </c>
+      <c r="C207">
+        <v>24</v>
+      </c>
+      <c r="D207">
+        <v>7186.490000000001</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>07/26</v>
+      </c>
+      <c r="B208">
+        <v>244.29899999999998</v>
+      </c>
+      <c r="C208">
+        <v>10</v>
+      </c>
+      <c r="D208">
+        <v>2442.99</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D194"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D208"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Promised Land Cloudbeds export from Drive — 2026-08-03
</commit_message>
<xml_diff>
--- a/PA-PL_occupancy_2026ytd.xlsx
+++ b/PA-PL_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D208"/>
+  <dimension ref="A1:D215"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1608,13 +1608,13 @@
         <v>03/27</v>
       </c>
       <c r="B87">
-        <v>181.83999999999997</v>
+        <v>181.84</v>
       </c>
       <c r="C87">
         <v>5</v>
       </c>
       <c r="D87">
-        <v>909.1999999999999</v>
+        <v>909.2</v>
       </c>
     </row>
     <row r="88">
@@ -1902,13 +1902,13 @@
         <v>04/17</v>
       </c>
       <c r="B108">
-        <v>210.77142857142857</v>
+        <v>210.77142857142854</v>
       </c>
       <c r="C108">
         <v>14</v>
       </c>
       <c r="D108">
-        <v>2950.8</v>
+        <v>2950.7999999999997</v>
       </c>
     </row>
     <row r="109">
@@ -2000,13 +2000,13 @@
         <v>04/24</v>
       </c>
       <c r="B115">
-        <v>206.55000000000004</v>
+        <v>206.54999999999998</v>
       </c>
       <c r="C115">
         <v>12</v>
       </c>
       <c r="D115">
-        <v>2478.6000000000004</v>
+        <v>2478.6</v>
       </c>
     </row>
     <row r="116">
@@ -2014,13 +2014,13 @@
         <v>04/25</v>
       </c>
       <c r="B116">
-        <v>212.13846153846154</v>
+        <v>212.1384615384615</v>
       </c>
       <c r="C116">
         <v>13</v>
       </c>
       <c r="D116">
-        <v>2757.8</v>
+        <v>2757.7999999999997</v>
       </c>
     </row>
     <row r="117">
@@ -2098,13 +2098,13 @@
         <v>05/01</v>
       </c>
       <c r="B122">
-        <v>238.5</v>
+        <v>238.49999999999997</v>
       </c>
       <c r="C122">
         <v>13</v>
       </c>
       <c r="D122">
-        <v>3100.5</v>
+        <v>3100.4999999999995</v>
       </c>
     </row>
     <row r="123">
@@ -2294,13 +2294,13 @@
         <v>05/15</v>
       </c>
       <c r="B136">
-        <v>287.18666666666667</v>
+        <v>287.1866666666667</v>
       </c>
       <c r="C136">
         <v>15</v>
       </c>
       <c r="D136">
-        <v>4307.8</v>
+        <v>4307.800000000001</v>
       </c>
     </row>
     <row r="137">
@@ -2398,7 +2398,7 @@
         <v>12</v>
       </c>
       <c r="D143">
-        <v>3448.4500000000003</v>
+        <v>3448.45</v>
       </c>
     </row>
     <row r="144">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>283.97772727272724</v>
+        <v>283.9777272727272</v>
       </c>
       <c r="C144">
         <v>22</v>
       </c>
       <c r="D144">
-        <v>6247.509999999999</v>
+        <v>6247.509999999998</v>
       </c>
     </row>
     <row r="145">
@@ -2518,13 +2518,13 @@
         <v>05/31</v>
       </c>
       <c r="B152">
-        <v>209.8222222222222</v>
+        <v>209.82222222222222</v>
       </c>
       <c r="C152">
         <v>9</v>
       </c>
       <c r="D152">
-        <v>1888.3999999999999</v>
+        <v>1888.4</v>
       </c>
     </row>
     <row r="153">
@@ -2588,13 +2588,13 @@
         <v>06/05</v>
       </c>
       <c r="B157">
-        <v>253.39499999999995</v>
+        <v>253.39499999999998</v>
       </c>
       <c r="C157">
         <v>16</v>
       </c>
       <c r="D157">
-        <v>4054.3199999999993</v>
+        <v>4054.3199999999997</v>
       </c>
     </row>
     <row r="158">
@@ -2686,13 +2686,13 @@
         <v>06/12</v>
       </c>
       <c r="B164">
-        <v>268.8158823529412</v>
+        <v>268.81588235294123</v>
       </c>
       <c r="C164">
         <v>17</v>
       </c>
       <c r="D164">
-        <v>4569.87</v>
+        <v>4569.870000000001</v>
       </c>
     </row>
     <row r="165">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>276.4234782608696</v>
+        <v>276.42347826086956</v>
       </c>
       <c r="C165">
         <v>23</v>
       </c>
       <c r="D165">
-        <v>6357.740000000001</v>
+        <v>6357.74</v>
       </c>
     </row>
     <row r="166">
@@ -2812,13 +2812,13 @@
         <v>06/21</v>
       </c>
       <c r="B173">
-        <v>199.6533333333333</v>
+        <v>199.65333333333334</v>
       </c>
       <c r="C173">
         <v>15</v>
       </c>
       <c r="D173">
-        <v>2994.7999999999997</v>
+        <v>2994.8</v>
       </c>
     </row>
     <row r="174">
@@ -2840,13 +2840,13 @@
         <v>06/23</v>
       </c>
       <c r="B175">
-        <v>232.02333333333334</v>
+        <v>232.0233333333333</v>
       </c>
       <c r="C175">
         <v>6</v>
       </c>
       <c r="D175">
-        <v>1392.14</v>
+        <v>1392.1399999999999</v>
       </c>
     </row>
     <row r="176">
@@ -2966,13 +2966,13 @@
         <v>07/02</v>
       </c>
       <c r="B184">
-        <v>346.905</v>
+        <v>346.90500000000003</v>
       </c>
       <c r="C184">
         <v>6</v>
       </c>
       <c r="D184">
-        <v>2081.43</v>
+        <v>2081.4300000000003</v>
       </c>
     </row>
     <row r="185">
@@ -3008,13 +3008,13 @@
         <v>07/05</v>
       </c>
       <c r="B187">
-        <v>218.89300000000003</v>
+        <v>218.89299999999997</v>
       </c>
       <c r="C187">
         <v>10</v>
       </c>
       <c r="D187">
-        <v>2188.9300000000003</v>
+        <v>2188.93</v>
       </c>
     </row>
     <row r="188">
@@ -3036,13 +3036,13 @@
         <v>07/07</v>
       </c>
       <c r="B189">
-        <v>213.58499999999998</v>
+        <v>213.58500000000004</v>
       </c>
       <c r="C189">
         <v>10</v>
       </c>
       <c r="D189">
-        <v>2135.85</v>
+        <v>2135.8500000000004</v>
       </c>
     </row>
     <row r="190">
@@ -3204,13 +3204,13 @@
         <v>07/19</v>
       </c>
       <c r="B201">
-        <v>269.0576923076923</v>
+        <v>269.05769230769226</v>
       </c>
       <c r="C201">
         <v>13</v>
       </c>
       <c r="D201">
-        <v>3497.75</v>
+        <v>3497.7499999999995</v>
       </c>
     </row>
     <row r="202">
@@ -3288,13 +3288,13 @@
         <v>07/25</v>
       </c>
       <c r="B207">
-        <v>299.43708333333336</v>
+        <v>299.4370833333333</v>
       </c>
       <c r="C207">
         <v>24</v>
       </c>
       <c r="D207">
-        <v>7186.490000000001</v>
+        <v>7186.49</v>
       </c>
     </row>
     <row r="208">
@@ -3311,9 +3311,107 @@
         <v>2442.99</v>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>07/27</v>
+      </c>
+      <c r="B209">
+        <v>262.392</v>
+      </c>
+      <c r="C209">
+        <v>10</v>
+      </c>
+      <c r="D209">
+        <v>2623.92</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>07/28</v>
+      </c>
+      <c r="B210">
+        <v>258.26599999999996</v>
+      </c>
+      <c r="C210">
+        <v>5</v>
+      </c>
+      <c r="D210">
+        <v>1291.33</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>07/29</v>
+      </c>
+      <c r="B211">
+        <v>255.55777777777777</v>
+      </c>
+      <c r="C211">
+        <v>9</v>
+      </c>
+      <c r="D211">
+        <v>2300.02</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>07/30</v>
+      </c>
+      <c r="B212">
+        <v>284.473</v>
+      </c>
+      <c r="C212">
+        <v>10</v>
+      </c>
+      <c r="D212">
+        <v>2844.73</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>07/31</v>
+      </c>
+      <c r="B213">
+        <v>315.41625</v>
+      </c>
+      <c r="C213">
+        <v>24</v>
+      </c>
+      <c r="D213">
+        <v>7569.99</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>08/01</v>
+      </c>
+      <c r="B214">
+        <v>345.70875</v>
+      </c>
+      <c r="C214">
+        <v>24</v>
+      </c>
+      <c r="D214">
+        <v>8297.01</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>08/02</v>
+      </c>
+      <c r="B215">
+        <v>340.75</v>
+      </c>
+      <c r="C215">
+        <v>8</v>
+      </c>
+      <c r="D215">
+        <v>2726</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D208"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D215"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Promised Land Cloudbeds export from Drive — 2026-08-11
</commit_message>
<xml_diff>
--- a/PA-PL_occupancy_2026ytd.xlsx
+++ b/PA-PL_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D215"/>
+  <dimension ref="A1:D222"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,13 +432,13 @@
         <v>01/02</v>
       </c>
       <c r="B3">
-        <v>275.09749999999997</v>
+        <v>275.0975</v>
       </c>
       <c r="C3">
         <v>4</v>
       </c>
       <c r="D3">
-        <v>1100.3899999999999</v>
+        <v>1100.39</v>
       </c>
     </row>
     <row r="4">
@@ -642,13 +642,13 @@
         <v>01/17</v>
       </c>
       <c r="B18">
-        <v>300.96666666666664</v>
+        <v>300.9666666666667</v>
       </c>
       <c r="C18">
         <v>6</v>
       </c>
       <c r="D18">
-        <v>1805.8</v>
+        <v>1805.8000000000002</v>
       </c>
     </row>
     <row r="19">
@@ -1048,13 +1048,13 @@
         <v>02/15</v>
       </c>
       <c r="B47">
-        <v>326.59833333333336</v>
+        <v>326.5983333333333</v>
       </c>
       <c r="C47">
         <v>6</v>
       </c>
       <c r="D47">
-        <v>1959.5900000000001</v>
+        <v>1959.59</v>
       </c>
     </row>
     <row r="48">
@@ -1132,13 +1132,13 @@
         <v>02/21</v>
       </c>
       <c r="B53">
-        <v>266.46799999999996</v>
+        <v>266.468</v>
       </c>
       <c r="C53">
         <v>5</v>
       </c>
       <c r="D53">
-        <v>1332.34</v>
+        <v>1332.3400000000001</v>
       </c>
     </row>
     <row r="54">
@@ -1412,13 +1412,13 @@
         <v>03/13</v>
       </c>
       <c r="B73">
-        <v>200.86999999999998</v>
+        <v>200.87</v>
       </c>
       <c r="C73">
         <v>6</v>
       </c>
       <c r="D73">
-        <v>1205.2199999999998</v>
+        <v>1205.22</v>
       </c>
     </row>
     <row r="74">
@@ -2098,13 +2098,13 @@
         <v>05/01</v>
       </c>
       <c r="B122">
-        <v>238.49999999999997</v>
+        <v>238.5</v>
       </c>
       <c r="C122">
         <v>13</v>
       </c>
       <c r="D122">
-        <v>3100.4999999999995</v>
+        <v>3100.5</v>
       </c>
     </row>
     <row r="123">
@@ -2112,13 +2112,13 @@
         <v>05/02</v>
       </c>
       <c r="B123">
-        <v>236.94285714285712</v>
+        <v>236.94285714285715</v>
       </c>
       <c r="C123">
         <v>14</v>
       </c>
       <c r="D123">
-        <v>3317.2</v>
+        <v>3317.2000000000003</v>
       </c>
     </row>
     <row r="124">
@@ -2266,13 +2266,13 @@
         <v>05/13</v>
       </c>
       <c r="B134">
-        <v>162.9333333333333</v>
+        <v>162.93333333333334</v>
       </c>
       <c r="C134">
         <v>3</v>
       </c>
       <c r="D134">
-        <v>488.79999999999995</v>
+        <v>488.8</v>
       </c>
     </row>
     <row r="135">
@@ -2322,13 +2322,13 @@
         <v>05/17</v>
       </c>
       <c r="B138">
-        <v>187.575</v>
+        <v>187.57500000000002</v>
       </c>
       <c r="C138">
         <v>8</v>
       </c>
       <c r="D138">
-        <v>1500.6</v>
+        <v>1500.6000000000001</v>
       </c>
     </row>
     <row r="139">
@@ -2350,13 +2350,13 @@
         <v>05/19</v>
       </c>
       <c r="B140">
-        <v>141.27499999999998</v>
+        <v>141.275</v>
       </c>
       <c r="C140">
         <v>8</v>
       </c>
       <c r="D140">
-        <v>1130.1999999999998</v>
+        <v>1130.2</v>
       </c>
     </row>
     <row r="141">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>283.9777272727272</v>
+        <v>283.97772727272724</v>
       </c>
       <c r="C144">
         <v>22</v>
       </c>
       <c r="D144">
-        <v>6247.509999999998</v>
+        <v>6247.509999999999</v>
       </c>
     </row>
     <row r="145">
@@ -2420,13 +2420,13 @@
         <v>05/24</v>
       </c>
       <c r="B145">
-        <v>294.62590909090903</v>
+        <v>294.6259090909091</v>
       </c>
       <c r="C145">
         <v>22</v>
       </c>
       <c r="D145">
-        <v>6481.769999999999</v>
+        <v>6481.7699999999995</v>
       </c>
     </row>
     <row r="146">
@@ -2504,13 +2504,13 @@
         <v>05/30</v>
       </c>
       <c r="B151">
-        <v>274.66764705882355</v>
+        <v>274.6676470588235</v>
       </c>
       <c r="C151">
         <v>17</v>
       </c>
       <c r="D151">
-        <v>4669.35</v>
+        <v>4669.349999999999</v>
       </c>
     </row>
     <row r="152">
@@ -2588,13 +2588,13 @@
         <v>06/05</v>
       </c>
       <c r="B157">
-        <v>253.39499999999998</v>
+        <v>253.39499999999995</v>
       </c>
       <c r="C157">
         <v>16</v>
       </c>
       <c r="D157">
-        <v>4054.3199999999997</v>
+        <v>4054.3199999999993</v>
       </c>
     </row>
     <row r="158">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>276.42347826086956</v>
+        <v>276.4234782608695</v>
       </c>
       <c r="C165">
         <v>23</v>
       </c>
       <c r="D165">
-        <v>6357.74</v>
+        <v>6357.739999999999</v>
       </c>
     </row>
     <row r="166">
@@ -2804,7 +2804,7 @@
         <v>19</v>
       </c>
       <c r="D172">
-        <v>6173.469999999999</v>
+        <v>6173.47</v>
       </c>
     </row>
     <row r="173">
@@ -2966,13 +2966,13 @@
         <v>07/02</v>
       </c>
       <c r="B184">
-        <v>346.90500000000003</v>
+        <v>346.905</v>
       </c>
       <c r="C184">
         <v>6</v>
       </c>
       <c r="D184">
-        <v>2081.4300000000003</v>
+        <v>2081.43</v>
       </c>
     </row>
     <row r="185">
@@ -3008,13 +3008,13 @@
         <v>07/05</v>
       </c>
       <c r="B187">
-        <v>218.89299999999997</v>
+        <v>218.89300000000003</v>
       </c>
       <c r="C187">
         <v>10</v>
       </c>
       <c r="D187">
-        <v>2188.93</v>
+        <v>2188.9300000000003</v>
       </c>
     </row>
     <row r="188">
@@ -3106,13 +3106,13 @@
         <v>07/12</v>
       </c>
       <c r="B194">
-        <v>250.16125</v>
+        <v>250.16125000000002</v>
       </c>
       <c r="C194">
         <v>8</v>
       </c>
       <c r="D194">
-        <v>2001.29</v>
+        <v>2001.2900000000002</v>
       </c>
     </row>
     <row r="195">
@@ -3176,13 +3176,13 @@
         <v>07/17</v>
       </c>
       <c r="B199">
-        <v>318.5835294117647</v>
+        <v>318.58352941176463</v>
       </c>
       <c r="C199">
         <v>17</v>
       </c>
       <c r="D199">
-        <v>5415.92</v>
+        <v>5415.919999999999</v>
       </c>
     </row>
     <row r="200">
@@ -3190,13 +3190,13 @@
         <v>07/18</v>
       </c>
       <c r="B200">
-        <v>311.26523809523815</v>
+        <v>311.2652380952381</v>
       </c>
       <c r="C200">
         <v>21</v>
       </c>
       <c r="D200">
-        <v>6536.570000000001</v>
+        <v>6536.57</v>
       </c>
     </row>
     <row r="201">
@@ -3204,13 +3204,13 @@
         <v>07/19</v>
       </c>
       <c r="B201">
-        <v>269.05769230769226</v>
+        <v>269.0576923076923</v>
       </c>
       <c r="C201">
         <v>13</v>
       </c>
       <c r="D201">
-        <v>3497.7499999999995</v>
+        <v>3497.75</v>
       </c>
     </row>
     <row r="202">
@@ -3224,7 +3224,7 @@
         <v>9</v>
       </c>
       <c r="D202">
-        <v>2363.2</v>
+        <v>2363.2000000000003</v>
       </c>
     </row>
     <row r="203">
@@ -3260,13 +3260,13 @@
         <v>07/23</v>
       </c>
       <c r="B205">
-        <v>227.63666666666668</v>
+        <v>227.63666666666666</v>
       </c>
       <c r="C205">
         <v>6</v>
       </c>
       <c r="D205">
-        <v>1365.8200000000002</v>
+        <v>1365.82</v>
       </c>
     </row>
     <row r="206">
@@ -3294,7 +3294,7 @@
         <v>24</v>
       </c>
       <c r="D207">
-        <v>7186.49</v>
+        <v>7186.489999999999</v>
       </c>
     </row>
     <row r="208">
@@ -3372,13 +3372,13 @@
         <v>07/31</v>
       </c>
       <c r="B213">
-        <v>315.41625</v>
+        <v>315.41624999999993</v>
       </c>
       <c r="C213">
         <v>24</v>
       </c>
       <c r="D213">
-        <v>7569.99</v>
+        <v>7569.989999999999</v>
       </c>
     </row>
     <row r="214">
@@ -3409,9 +3409,107 @@
         <v>2726</v>
       </c>
     </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>08/03</v>
+      </c>
+      <c r="B216">
+        <v>259.28499999999997</v>
+      </c>
+      <c r="C216">
+        <v>14</v>
+      </c>
+      <c r="D216">
+        <v>3629.99</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>08/04</v>
+      </c>
+      <c r="B217">
+        <v>252.19538461538463</v>
+      </c>
+      <c r="C217">
+        <v>13</v>
+      </c>
+      <c r="D217">
+        <v>3278.54</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>08/05</v>
+      </c>
+      <c r="B218">
+        <v>256.10833333333335</v>
+      </c>
+      <c r="C218">
+        <v>6</v>
+      </c>
+      <c r="D218">
+        <v>1536.65</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>08/06</v>
+      </c>
+      <c r="B219">
+        <v>223.6575</v>
+      </c>
+      <c r="C219">
+        <v>4</v>
+      </c>
+      <c r="D219">
+        <v>894.63</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>08/07</v>
+      </c>
+      <c r="B220">
+        <v>345.05058823529413</v>
+      </c>
+      <c r="C220">
+        <v>17</v>
+      </c>
+      <c r="D220">
+        <v>5865.860000000001</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>08/08</v>
+      </c>
+      <c r="B221">
+        <v>343.19541666666674</v>
+      </c>
+      <c r="C221">
+        <v>24</v>
+      </c>
+      <c r="D221">
+        <v>8236.690000000002</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>08/09</v>
+      </c>
+      <c r="B222">
+        <v>273.3617391304348</v>
+      </c>
+      <c r="C222">
+        <v>23</v>
+      </c>
+      <c r="D222">
+        <v>6287.32</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D215"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D222"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Promised Land Cloudbeds export from Drive — 2026-08-17
</commit_message>
<xml_diff>
--- a/PA-PL_occupancy_2026ytd.xlsx
+++ b/PA-PL_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D222"/>
+  <dimension ref="A1:D230"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,13 +432,13 @@
         <v>01/02</v>
       </c>
       <c r="B3">
-        <v>275.0975</v>
+        <v>275.09749999999997</v>
       </c>
       <c r="C3">
         <v>4</v>
       </c>
       <c r="D3">
-        <v>1100.39</v>
+        <v>1100.3899999999999</v>
       </c>
     </row>
     <row r="4">
@@ -572,13 +572,13 @@
         <v>01/12</v>
       </c>
       <c r="B13">
-        <v>122.93333333333332</v>
+        <v>122.93333333333334</v>
       </c>
       <c r="C13">
         <v>3</v>
       </c>
       <c r="D13">
-        <v>368.79999999999995</v>
+        <v>368.8</v>
       </c>
     </row>
     <row r="14">
@@ -1124,7 +1124,7 @@
         <v>5</v>
       </c>
       <c r="D52">
-        <v>1290.65</v>
+        <v>1290.6499999999999</v>
       </c>
     </row>
     <row r="53">
@@ -1230,13 +1230,13 @@
         <v>02/28</v>
       </c>
       <c r="B60">
-        <v>239.0533333333333</v>
+        <v>239.05333333333337</v>
       </c>
       <c r="C60">
         <v>6</v>
       </c>
       <c r="D60">
-        <v>1434.32</v>
+        <v>1434.3200000000002</v>
       </c>
     </row>
     <row r="61">
@@ -1510,13 +1510,13 @@
         <v>03/20</v>
       </c>
       <c r="B80">
-        <v>195.98000000000002</v>
+        <v>195.98</v>
       </c>
       <c r="C80">
         <v>6</v>
       </c>
       <c r="D80">
-        <v>1175.88</v>
+        <v>1175.8799999999999</v>
       </c>
     </row>
     <row r="81">
@@ -1608,13 +1608,13 @@
         <v>03/27</v>
       </c>
       <c r="B87">
-        <v>181.84</v>
+        <v>181.83999999999997</v>
       </c>
       <c r="C87">
         <v>5</v>
       </c>
       <c r="D87">
-        <v>909.2</v>
+        <v>909.1999999999999</v>
       </c>
     </row>
     <row r="88">
@@ -2000,13 +2000,13 @@
         <v>04/24</v>
       </c>
       <c r="B115">
-        <v>206.54999999999998</v>
+        <v>206.55000000000004</v>
       </c>
       <c r="C115">
         <v>12</v>
       </c>
       <c r="D115">
-        <v>2478.6</v>
+        <v>2478.6000000000004</v>
       </c>
     </row>
     <row r="116">
@@ -2266,13 +2266,13 @@
         <v>05/13</v>
       </c>
       <c r="B134">
-        <v>162.93333333333334</v>
+        <v>162.9333333333333</v>
       </c>
       <c r="C134">
         <v>3</v>
       </c>
       <c r="D134">
-        <v>488.8</v>
+        <v>488.79999999999995</v>
       </c>
     </row>
     <row r="135">
@@ -2294,13 +2294,13 @@
         <v>05/15</v>
       </c>
       <c r="B136">
-        <v>287.1866666666667</v>
+        <v>287.18666666666667</v>
       </c>
       <c r="C136">
         <v>15</v>
       </c>
       <c r="D136">
-        <v>4307.800000000001</v>
+        <v>4307.8</v>
       </c>
     </row>
     <row r="137">
@@ -2336,13 +2336,13 @@
         <v>05/18</v>
       </c>
       <c r="B139">
-        <v>151.62857142857143</v>
+        <v>151.6285714285714</v>
       </c>
       <c r="C139">
         <v>7</v>
       </c>
       <c r="D139">
-        <v>1061.4</v>
+        <v>1061.3999999999999</v>
       </c>
     </row>
     <row r="140">
@@ -2364,13 +2364,13 @@
         <v>05/20</v>
       </c>
       <c r="B141">
-        <v>147.25714285714284</v>
+        <v>147.2571428571429</v>
       </c>
       <c r="C141">
         <v>7</v>
       </c>
       <c r="D141">
-        <v>1030.8</v>
+        <v>1030.8000000000002</v>
       </c>
     </row>
     <row r="142">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>283.97772727272724</v>
+        <v>283.9777272727272</v>
       </c>
       <c r="C144">
         <v>22</v>
       </c>
       <c r="D144">
-        <v>6247.509999999999</v>
+        <v>6247.509999999998</v>
       </c>
     </row>
     <row r="145">
@@ -2420,13 +2420,13 @@
         <v>05/24</v>
       </c>
       <c r="B145">
-        <v>294.6259090909091</v>
+        <v>294.62590909090903</v>
       </c>
       <c r="C145">
         <v>22</v>
       </c>
       <c r="D145">
-        <v>6481.7699999999995</v>
+        <v>6481.769999999999</v>
       </c>
     </row>
     <row r="146">
@@ -2504,13 +2504,13 @@
         <v>05/30</v>
       </c>
       <c r="B151">
-        <v>274.6676470588235</v>
+        <v>274.66764705882355</v>
       </c>
       <c r="C151">
         <v>17</v>
       </c>
       <c r="D151">
-        <v>4669.349999999999</v>
+        <v>4669.35</v>
       </c>
     </row>
     <row r="152">
@@ -2588,13 +2588,13 @@
         <v>06/05</v>
       </c>
       <c r="B157">
-        <v>253.39499999999995</v>
+        <v>253.39499999999998</v>
       </c>
       <c r="C157">
         <v>16</v>
       </c>
       <c r="D157">
-        <v>4054.3199999999993</v>
+        <v>4054.3199999999997</v>
       </c>
     </row>
     <row r="158">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>276.4234782608695</v>
+        <v>276.42347826086956</v>
       </c>
       <c r="C165">
         <v>23</v>
       </c>
       <c r="D165">
-        <v>6357.739999999999</v>
+        <v>6357.74</v>
       </c>
     </row>
     <row r="166">
@@ -2714,13 +2714,13 @@
         <v>06/14</v>
       </c>
       <c r="B166">
-        <v>224.3183333333333</v>
+        <v>224.31833333333336</v>
       </c>
       <c r="C166">
         <v>6</v>
       </c>
       <c r="D166">
-        <v>1345.9099999999999</v>
+        <v>1345.91</v>
       </c>
     </row>
     <row r="167">
@@ -2840,13 +2840,13 @@
         <v>06/23</v>
       </c>
       <c r="B175">
-        <v>232.0233333333333</v>
+        <v>232.02333333333334</v>
       </c>
       <c r="C175">
         <v>6</v>
       </c>
       <c r="D175">
-        <v>1392.1399999999999</v>
+        <v>1392.14</v>
       </c>
     </row>
     <row r="176">
@@ -2896,13 +2896,13 @@
         <v>06/27</v>
       </c>
       <c r="B179">
-        <v>305.48545454545456</v>
+        <v>305.4854545454545</v>
       </c>
       <c r="C179">
         <v>22</v>
       </c>
       <c r="D179">
-        <v>6720.68</v>
+        <v>6720.679999999999</v>
       </c>
     </row>
     <row r="180">
@@ -2966,13 +2966,13 @@
         <v>07/02</v>
       </c>
       <c r="B184">
-        <v>346.905</v>
+        <v>346.90500000000003</v>
       </c>
       <c r="C184">
         <v>6</v>
       </c>
       <c r="D184">
-        <v>2081.43</v>
+        <v>2081.4300000000003</v>
       </c>
     </row>
     <row r="185">
@@ -3036,13 +3036,13 @@
         <v>07/07</v>
       </c>
       <c r="B189">
-        <v>213.58500000000004</v>
+        <v>213.58499999999998</v>
       </c>
       <c r="C189">
         <v>10</v>
       </c>
       <c r="D189">
-        <v>2135.8500000000004</v>
+        <v>2135.85</v>
       </c>
     </row>
     <row r="190">
@@ -3092,13 +3092,13 @@
         <v>07/11</v>
       </c>
       <c r="B193">
-        <v>335.62952380952385</v>
+        <v>335.6295238095238</v>
       </c>
       <c r="C193">
         <v>21</v>
       </c>
       <c r="D193">
-        <v>7048.22</v>
+        <v>7048.219999999999</v>
       </c>
     </row>
     <row r="194">
@@ -3106,13 +3106,13 @@
         <v>07/12</v>
       </c>
       <c r="B194">
-        <v>250.16125000000002</v>
+        <v>250.16125</v>
       </c>
       <c r="C194">
         <v>8</v>
       </c>
       <c r="D194">
-        <v>2001.2900000000002</v>
+        <v>2001.29</v>
       </c>
     </row>
     <row r="195">
@@ -3294,7 +3294,7 @@
         <v>24</v>
       </c>
       <c r="D207">
-        <v>7186.489999999999</v>
+        <v>7186.49</v>
       </c>
     </row>
     <row r="208">
@@ -3372,13 +3372,13 @@
         <v>07/31</v>
       </c>
       <c r="B213">
-        <v>315.41624999999993</v>
+        <v>315.41625</v>
       </c>
       <c r="C213">
         <v>24</v>
       </c>
       <c r="D213">
-        <v>7569.989999999999</v>
+        <v>7569.99</v>
       </c>
     </row>
     <row r="214">
@@ -3386,13 +3386,13 @@
         <v>08/01</v>
       </c>
       <c r="B214">
-        <v>345.70875</v>
+        <v>345.70874999999995</v>
       </c>
       <c r="C214">
         <v>24</v>
       </c>
       <c r="D214">
-        <v>8297.01</v>
+        <v>8297.009999999998</v>
       </c>
     </row>
     <row r="215">
@@ -3470,13 +3470,13 @@
         <v>08/07</v>
       </c>
       <c r="B220">
-        <v>345.05058823529413</v>
+        <v>345.0505882352941</v>
       </c>
       <c r="C220">
         <v>17</v>
       </c>
       <c r="D220">
-        <v>5865.860000000001</v>
+        <v>5865.86</v>
       </c>
     </row>
     <row r="221">
@@ -3484,13 +3484,13 @@
         <v>08/08</v>
       </c>
       <c r="B221">
-        <v>343.19541666666674</v>
+        <v>334.0704166666667</v>
       </c>
       <c r="C221">
         <v>24</v>
       </c>
       <c r="D221">
-        <v>8236.690000000002</v>
+        <v>8017.6900000000005</v>
       </c>
     </row>
     <row r="222">
@@ -3498,18 +3498,130 @@
         <v>08/09</v>
       </c>
       <c r="B222">
-        <v>273.3617391304348</v>
+        <v>241.4534782608696</v>
       </c>
       <c r="C222">
         <v>23</v>
       </c>
       <c r="D222">
-        <v>6287.32</v>
+        <v>5553.43</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>08/10</v>
+      </c>
+      <c r="B223">
+        <v>250.20499999999998</v>
+      </c>
+      <c r="C223">
+        <v>10</v>
+      </c>
+      <c r="D223">
+        <v>2502.0499999999997</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>08/11</v>
+      </c>
+      <c r="B224">
+        <v>276.41333333333336</v>
+      </c>
+      <c r="C224">
+        <v>9</v>
+      </c>
+      <c r="D224">
+        <v>2487.7200000000003</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>08/12</v>
+      </c>
+      <c r="B225">
+        <v>243.06285714285715</v>
+      </c>
+      <c r="C225">
+        <v>7</v>
+      </c>
+      <c r="D225">
+        <v>1701.44</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>08/13</v>
+      </c>
+      <c r="B226">
+        <v>196.775</v>
+      </c>
+      <c r="C226">
+        <v>8</v>
+      </c>
+      <c r="D226">
+        <v>1574.2</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>08/14</v>
+      </c>
+      <c r="B227">
+        <v>300.6475</v>
+      </c>
+      <c r="C227">
+        <v>24</v>
+      </c>
+      <c r="D227">
+        <v>7215.54</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>08/15</v>
+      </c>
+      <c r="B228">
+        <v>304.7658333333333</v>
+      </c>
+      <c r="C228">
+        <v>24</v>
+      </c>
+      <c r="D228">
+        <v>7314.379999999999</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>08/16</v>
+      </c>
+      <c r="B229">
+        <v>242.855</v>
+      </c>
+      <c r="C229">
+        <v>14</v>
+      </c>
+      <c r="D229">
+        <v>3399.97</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>08/17</v>
+      </c>
+      <c r="B230">
+        <v>273.8828571428572</v>
+      </c>
+      <c r="C230">
+        <v>14</v>
+      </c>
+      <c r="D230">
+        <v>3834.36</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D222"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D230"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Promised Land Cloudbeds export from Drive — 2026-08-25
</commit_message>
<xml_diff>
--- a/PA-PL_occupancy_2026ytd.xlsx
+++ b/PA-PL_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D230"/>
+  <dimension ref="A1:D236"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -642,13 +642,13 @@
         <v>01/17</v>
       </c>
       <c r="B18">
-        <v>300.9666666666667</v>
+        <v>300.96666666666664</v>
       </c>
       <c r="C18">
         <v>6</v>
       </c>
       <c r="D18">
-        <v>1805.8000000000002</v>
+        <v>1805.8</v>
       </c>
     </row>
     <row r="19">
@@ -1132,13 +1132,13 @@
         <v>02/21</v>
       </c>
       <c r="B53">
-        <v>266.468</v>
+        <v>266.46799999999996</v>
       </c>
       <c r="C53">
         <v>5</v>
       </c>
       <c r="D53">
-        <v>1332.3400000000001</v>
+        <v>1332.34</v>
       </c>
     </row>
     <row r="54">
@@ -1230,13 +1230,13 @@
         <v>02/28</v>
       </c>
       <c r="B60">
-        <v>239.05333333333337</v>
+        <v>239.0533333333333</v>
       </c>
       <c r="C60">
         <v>6</v>
       </c>
       <c r="D60">
-        <v>1434.3200000000002</v>
+        <v>1434.32</v>
       </c>
     </row>
     <row r="61">
@@ -1412,13 +1412,13 @@
         <v>03/13</v>
       </c>
       <c r="B73">
-        <v>200.87</v>
+        <v>200.86999999999998</v>
       </c>
       <c r="C73">
         <v>6</v>
       </c>
       <c r="D73">
-        <v>1205.22</v>
+        <v>1205.2199999999998</v>
       </c>
     </row>
     <row r="74">
@@ -1608,13 +1608,13 @@
         <v>03/27</v>
       </c>
       <c r="B87">
-        <v>181.83999999999997</v>
+        <v>181.84</v>
       </c>
       <c r="C87">
         <v>5</v>
       </c>
       <c r="D87">
-        <v>909.1999999999999</v>
+        <v>909.2</v>
       </c>
     </row>
     <row r="88">
@@ -1902,13 +1902,13 @@
         <v>04/17</v>
       </c>
       <c r="B108">
-        <v>210.77142857142854</v>
+        <v>210.77142857142857</v>
       </c>
       <c r="C108">
         <v>14</v>
       </c>
       <c r="D108">
-        <v>2950.7999999999997</v>
+        <v>2950.8</v>
       </c>
     </row>
     <row r="109">
@@ -2014,13 +2014,13 @@
         <v>04/25</v>
       </c>
       <c r="B116">
-        <v>212.1384615384615</v>
+        <v>212.13846153846154</v>
       </c>
       <c r="C116">
         <v>13</v>
       </c>
       <c r="D116">
-        <v>2757.7999999999997</v>
+        <v>2757.8</v>
       </c>
     </row>
     <row r="117">
@@ -2098,13 +2098,13 @@
         <v>05/01</v>
       </c>
       <c r="B122">
-        <v>238.5</v>
+        <v>238.49999999999997</v>
       </c>
       <c r="C122">
         <v>13</v>
       </c>
       <c r="D122">
-        <v>3100.5</v>
+        <v>3100.4999999999995</v>
       </c>
     </row>
     <row r="123">
@@ -2112,13 +2112,13 @@
         <v>05/02</v>
       </c>
       <c r="B123">
-        <v>236.94285714285715</v>
+        <v>236.9428571428572</v>
       </c>
       <c r="C123">
         <v>14</v>
       </c>
       <c r="D123">
-        <v>3317.2000000000003</v>
+        <v>3317.2000000000007</v>
       </c>
     </row>
     <row r="124">
@@ -2336,13 +2336,13 @@
         <v>05/18</v>
       </c>
       <c r="B139">
-        <v>151.6285714285714</v>
+        <v>151.62857142857143</v>
       </c>
       <c r="C139">
         <v>7</v>
       </c>
       <c r="D139">
-        <v>1061.3999999999999</v>
+        <v>1061.4</v>
       </c>
     </row>
     <row r="140">
@@ -2364,13 +2364,13 @@
         <v>05/20</v>
       </c>
       <c r="B141">
-        <v>147.2571428571429</v>
+        <v>147.25714285714284</v>
       </c>
       <c r="C141">
         <v>7</v>
       </c>
       <c r="D141">
-        <v>1030.8000000000002</v>
+        <v>1030.8</v>
       </c>
     </row>
     <row r="142">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>283.9777272727272</v>
+        <v>283.97772727272724</v>
       </c>
       <c r="C144">
         <v>22</v>
       </c>
       <c r="D144">
-        <v>6247.509999999998</v>
+        <v>6247.509999999999</v>
       </c>
     </row>
     <row r="145">
@@ -2434,13 +2434,13 @@
         <v>05/25</v>
       </c>
       <c r="B146">
-        <v>177.4811111111111</v>
+        <v>177.48111111111112</v>
       </c>
       <c r="C146">
         <v>9</v>
       </c>
       <c r="D146">
-        <v>1597.33</v>
+        <v>1597.3300000000002</v>
       </c>
     </row>
     <row r="147">
@@ -2686,13 +2686,13 @@
         <v>06/12</v>
       </c>
       <c r="B164">
-        <v>268.81588235294123</v>
+        <v>268.8158823529412</v>
       </c>
       <c r="C164">
         <v>17</v>
       </c>
       <c r="D164">
-        <v>4569.870000000001</v>
+        <v>4569.87</v>
       </c>
     </row>
     <row r="165">
@@ -2784,13 +2784,13 @@
         <v>06/19</v>
       </c>
       <c r="B171">
-        <v>305.4868421052632</v>
+        <v>305.4868421052631</v>
       </c>
       <c r="C171">
         <v>19</v>
       </c>
       <c r="D171">
-        <v>5804.25</v>
+        <v>5804.249999999999</v>
       </c>
     </row>
     <row r="172">
@@ -2804,7 +2804,7 @@
         <v>19</v>
       </c>
       <c r="D172">
-        <v>6173.47</v>
+        <v>6173.469999999999</v>
       </c>
     </row>
     <row r="173">
@@ -2812,13 +2812,13 @@
         <v>06/21</v>
       </c>
       <c r="B173">
-        <v>199.65333333333334</v>
+        <v>199.6533333333333</v>
       </c>
       <c r="C173">
         <v>15</v>
       </c>
       <c r="D173">
-        <v>2994.8</v>
+        <v>2994.7999999999997</v>
       </c>
     </row>
     <row r="174">
@@ -2840,13 +2840,13 @@
         <v>06/23</v>
       </c>
       <c r="B175">
-        <v>232.02333333333334</v>
+        <v>232.0233333333333</v>
       </c>
       <c r="C175">
         <v>6</v>
       </c>
       <c r="D175">
-        <v>1392.14</v>
+        <v>1392.1399999999999</v>
       </c>
     </row>
     <row r="176">
@@ -3036,13 +3036,13 @@
         <v>07/07</v>
       </c>
       <c r="B189">
-        <v>213.58499999999998</v>
+        <v>213.58500000000004</v>
       </c>
       <c r="C189">
         <v>10</v>
       </c>
       <c r="D189">
-        <v>2135.85</v>
+        <v>2135.8500000000004</v>
       </c>
     </row>
     <row r="190">
@@ -3134,13 +3134,13 @@
         <v>07/14</v>
       </c>
       <c r="B196">
-        <v>190.66750000000002</v>
+        <v>190.6675</v>
       </c>
       <c r="C196">
         <v>4</v>
       </c>
       <c r="D196">
-        <v>762.6700000000001</v>
+        <v>762.67</v>
       </c>
     </row>
     <row r="197">
@@ -3176,13 +3176,13 @@
         <v>07/17</v>
       </c>
       <c r="B199">
-        <v>318.58352941176463</v>
+        <v>318.5835294117647</v>
       </c>
       <c r="C199">
         <v>17</v>
       </c>
       <c r="D199">
-        <v>5415.919999999999</v>
+        <v>5415.92</v>
       </c>
     </row>
     <row r="200">
@@ -3190,13 +3190,13 @@
         <v>07/18</v>
       </c>
       <c r="B200">
-        <v>311.2652380952381</v>
+        <v>311.26523809523815</v>
       </c>
       <c r="C200">
         <v>21</v>
       </c>
       <c r="D200">
-        <v>6536.57</v>
+        <v>6536.570000000001</v>
       </c>
     </row>
     <row r="201">
@@ -3224,7 +3224,7 @@
         <v>9</v>
       </c>
       <c r="D202">
-        <v>2363.2000000000003</v>
+        <v>2363.2</v>
       </c>
     </row>
     <row r="203">
@@ -3260,13 +3260,13 @@
         <v>07/23</v>
       </c>
       <c r="B205">
-        <v>227.63666666666666</v>
+        <v>227.63666666666668</v>
       </c>
       <c r="C205">
         <v>6</v>
       </c>
       <c r="D205">
-        <v>1365.82</v>
+        <v>1365.8200000000002</v>
       </c>
     </row>
     <row r="206">
@@ -3288,13 +3288,13 @@
         <v>07/25</v>
       </c>
       <c r="B207">
-        <v>299.4370833333333</v>
+        <v>299.43708333333336</v>
       </c>
       <c r="C207">
         <v>24</v>
       </c>
       <c r="D207">
-        <v>7186.49</v>
+        <v>7186.490000000001</v>
       </c>
     </row>
     <row r="208">
@@ -3386,13 +3386,13 @@
         <v>08/01</v>
       </c>
       <c r="B214">
-        <v>345.70874999999995</v>
+        <v>345.70875</v>
       </c>
       <c r="C214">
         <v>24</v>
       </c>
       <c r="D214">
-        <v>8297.009999999998</v>
+        <v>8297.01</v>
       </c>
     </row>
     <row r="215">
@@ -3512,13 +3512,13 @@
         <v>08/10</v>
       </c>
       <c r="B223">
-        <v>250.20499999999998</v>
+        <v>250.205</v>
       </c>
       <c r="C223">
         <v>10</v>
       </c>
       <c r="D223">
-        <v>2502.0499999999997</v>
+        <v>2502.05</v>
       </c>
     </row>
     <row r="224">
@@ -3588,7 +3588,7 @@
         <v>24</v>
       </c>
       <c r="D228">
-        <v>7314.379999999999</v>
+        <v>7314.38</v>
       </c>
     </row>
     <row r="229">
@@ -3619,9 +3619,93 @@
         <v>3834.36</v>
       </c>
     </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>08/18</v>
+      </c>
+      <c r="B231">
+        <v>259.635294117647</v>
+      </c>
+      <c r="C231">
+        <v>17</v>
+      </c>
+      <c r="D231">
+        <v>4413.799999999999</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>08/19</v>
+      </c>
+      <c r="B232">
+        <v>223.78571428571428</v>
+      </c>
+      <c r="C232">
+        <v>21</v>
+      </c>
+      <c r="D232">
+        <v>4699.5</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>08/20</v>
+      </c>
+      <c r="B233">
+        <v>247.0090909090909</v>
+      </c>
+      <c r="C233">
+        <v>11</v>
+      </c>
+      <c r="D233">
+        <v>2717.1</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>08/21</v>
+      </c>
+      <c r="B234">
+        <v>306.76124999999996</v>
+      </c>
+      <c r="C234">
+        <v>24</v>
+      </c>
+      <c r="D234">
+        <v>7362.2699999999995</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>08/22</v>
+      </c>
+      <c r="B235">
+        <v>296.41260869565224</v>
+      </c>
+      <c r="C235">
+        <v>23</v>
+      </c>
+      <c r="D235">
+        <v>6817.490000000002</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>08/23</v>
+      </c>
+      <c r="B236">
+        <v>259.38176470588235</v>
+      </c>
+      <c r="C236">
+        <v>17</v>
+      </c>
+      <c r="D236">
+        <v>4409.49</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D230"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D236"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>